<commit_message>
updates adding new issues and removing outlier
</commit_message>
<xml_diff>
--- a/data/final/02_closed_issues_gsynth.xlsx
+++ b/data/final/02_closed_issues_gsynth.xlsx
@@ -394,19 +394,19 @@
         </is>
       </c>
       <c r="B2">
-        <v>-0.03428739448289855</v>
+        <v>-0.03428739448289302</v>
       </c>
       <c r="C2">
-        <v>0.5732516205624356</v>
+        <v>0.5882689427463792</v>
       </c>
       <c r="D2">
-        <v>0.060872132560657</v>
+        <v>0.06333727080210487</v>
       </c>
       <c r="E2">
-        <v>-0.1535945819639342</v>
+        <v>-0.1584261641340788</v>
       </c>
       <c r="F2">
-        <v>0.08501979299813706</v>
+        <v>0.08985137516829282</v>
       </c>
     </row>
     <row r="3">
@@ -416,19 +416,19 @@
         </is>
       </c>
       <c r="B3">
-        <v>-0.03119887116390507</v>
+        <v>-0.03119887116390258</v>
       </c>
       <c r="C3">
-        <v>0.60150576023891</v>
+        <v>0.6140946275113122</v>
       </c>
       <c r="D3">
-        <v>0.05974089983920539</v>
+        <v>0.06187338932396205</v>
       </c>
       <c r="E3">
-        <v>-0.1482888832527623</v>
+        <v>-0.1524684858402932</v>
       </c>
       <c r="F3">
-        <v>0.08589114092495216</v>
+        <v>0.09007074351248809</v>
       </c>
     </row>
     <row r="4">
@@ -438,19 +438,19 @@
         </is>
       </c>
       <c r="B4">
-        <v>0.02517237507600951</v>
+        <v>0.02517237507601412</v>
       </c>
       <c r="C4">
-        <v>0.6650411142421686</v>
+        <v>0.6700474543463286</v>
       </c>
       <c r="D4">
-        <v>0.0581396844498109</v>
+        <v>0.05907858831354344</v>
       </c>
       <c r="E4">
-        <v>-0.08877931251814324</v>
+        <v>-0.09061953027599992</v>
       </c>
       <c r="F4">
-        <v>0.1391240626701623</v>
+        <v>0.1409642804280282</v>
       </c>
     </row>
     <row r="5">
@@ -460,19 +460,19 @@
         </is>
       </c>
       <c r="B5">
-        <v>0.07837441317610375</v>
+        <v>0.07837441317610788</v>
       </c>
       <c r="C5">
-        <v>0.2105453321295812</v>
+        <v>0.2058528693100241</v>
       </c>
       <c r="D5">
-        <v>0.06259600542549479</v>
+        <v>0.06195353592328549</v>
       </c>
       <c r="E5">
-        <v>-0.04431150303393983</v>
+        <v>-0.04305228594844009</v>
       </c>
       <c r="F5">
-        <v>0.2010603293861473</v>
+        <v>0.1998011123006558</v>
       </c>
     </row>
     <row r="6">
@@ -482,19 +482,19 @@
         </is>
       </c>
       <c r="B6">
-        <v>-0.04776134130792694</v>
+        <v>-0.04776134130792607</v>
       </c>
       <c r="C6">
-        <v>0.4865996923228824</v>
+        <v>0.5047685495370418</v>
       </c>
       <c r="D6">
-        <v>0.0686495249540071</v>
+        <v>0.0716056065164897</v>
       </c>
       <c r="E6">
-        <v>-0.1823119377735645</v>
+        <v>-0.1881057511713924</v>
       </c>
       <c r="F6">
-        <v>0.08678925515771063</v>
+        <v>0.0925830685555403</v>
       </c>
     </row>
     <row r="7">
@@ -504,19 +504,19 @@
         </is>
       </c>
       <c r="B7">
-        <v>-0.06244970100523362</v>
+        <v>-0.06244970100523987</v>
       </c>
       <c r="C7">
-        <v>0.4220956839146484</v>
+        <v>0.4347341772628623</v>
       </c>
       <c r="D7">
-        <v>0.07779075712638502</v>
+        <v>0.07994931365507658</v>
       </c>
       <c r="E7">
-        <v>-0.2149167833030508</v>
+        <v>-0.2191474763578863</v>
       </c>
       <c r="F7">
-        <v>0.09001738129258352</v>
+        <v>0.09424807434740652</v>
       </c>
     </row>
     <row r="8">
@@ -526,19 +526,19 @@
         </is>
       </c>
       <c r="B8">
-        <v>-0.1490517950598902</v>
+        <v>-0.1490517950598938</v>
       </c>
       <c r="C8">
-        <v>0.1049544210109072</v>
+        <v>0.107099434987989</v>
       </c>
       <c r="D8">
-        <v>0.09193379965527873</v>
+        <v>0.09250013124872478</v>
       </c>
       <c r="E8">
-        <v>-0.3292387313461573</v>
+        <v>-0.3303487208726223</v>
       </c>
       <c r="F8">
-        <v>0.03113514122637687</v>
+        <v>0.03224513075283472</v>
       </c>
     </row>
     <row r="9">
@@ -548,19 +548,19 @@
         </is>
       </c>
       <c r="B9">
-        <v>-0.103287517542655</v>
+        <v>-0.1032875175426601</v>
       </c>
       <c r="C9">
-        <v>0.2890026646155901</v>
+        <v>0.2888281992249455</v>
       </c>
       <c r="D9">
-        <v>0.09741237850082438</v>
+        <v>0.09737714050411368</v>
       </c>
       <c r="E9">
-        <v>-0.2942122710526546</v>
+        <v>-0.2941432058482194</v>
       </c>
       <c r="F9">
-        <v>0.08763723596734456</v>
+        <v>0.08756817076289916</v>
       </c>
     </row>
     <row r="10">
@@ -570,19 +570,19 @@
         </is>
       </c>
       <c r="B10">
-        <v>0.02267066141720355</v>
+        <v>0.02267066141719816</v>
       </c>
       <c r="C10">
-        <v>0.699605113343545</v>
+        <v>0.6991276201702668</v>
       </c>
       <c r="D10">
-        <v>0.05875457108852128</v>
+        <v>0.05865655334572888</v>
       </c>
       <c r="E10">
-        <v>-0.09248618184339644</v>
+        <v>-0.09229407059768283</v>
       </c>
       <c r="F10">
-        <v>0.1378275046778035</v>
+        <v>0.1376353934320791</v>
       </c>
     </row>
     <row r="11">
@@ -592,19 +592,19 @@
         </is>
       </c>
       <c r="B11">
-        <v>0.08366826570735021</v>
+        <v>0.08366826570733929</v>
       </c>
       <c r="C11">
-        <v>0.2929578035430587</v>
+        <v>0.2989329208446101</v>
       </c>
       <c r="D11">
-        <v>0.07955865301211856</v>
+        <v>0.08054905048934131</v>
       </c>
       <c r="E11">
-        <v>-0.07226382885492121</v>
+        <v>-0.07420497224066805</v>
       </c>
       <c r="F11">
-        <v>0.2396003602696216</v>
+        <v>0.2415415036553466</v>
       </c>
     </row>
     <row r="12">
@@ -614,19 +614,19 @@
         </is>
       </c>
       <c r="B12">
-        <v>0.03534921683207792</v>
+        <v>0.035349216832072</v>
       </c>
       <c r="C12">
-        <v>0.560863383181327</v>
+        <v>0.5564276414844684</v>
       </c>
       <c r="D12">
-        <v>0.06078348416177968</v>
+        <v>0.06010177850179366</v>
       </c>
       <c r="E12">
-        <v>-0.08378422297987101</v>
+        <v>-0.08244810443824722</v>
       </c>
       <c r="F12">
-        <v>0.1544826566440269</v>
+        <v>0.1531465381023912</v>
       </c>
     </row>
     <row r="13">
@@ -636,19 +636,19 @@
         </is>
       </c>
       <c r="B13">
-        <v>0.0990637652302767</v>
+        <v>0.09906376523027875</v>
       </c>
       <c r="C13">
-        <v>0.1147204420458716</v>
+        <v>0.1216126914328732</v>
       </c>
       <c r="D13">
-        <v>0.0628048611591092</v>
+        <v>0.06399303113016447</v>
       </c>
       <c r="E13">
-        <v>-0.02403150069561581</v>
+        <v>-0.02636027104639409</v>
       </c>
       <c r="F13">
-        <v>0.2221590311561692</v>
+        <v>0.2244878015069516</v>
       </c>
     </row>
     <row r="14">
@@ -658,19 +658,19 @@
         </is>
       </c>
       <c r="B14">
-        <v>0.2036332504646791</v>
+        <v>0.2036332504646786</v>
       </c>
       <c r="C14">
-        <v>0.006119763297230518</v>
+        <v>0.008264179492954993</v>
       </c>
       <c r="D14">
-        <v>0.07428361024380979</v>
+        <v>0.0771022163704871</v>
       </c>
       <c r="E14">
-        <v>0.05804004974520138</v>
+        <v>0.05251568325030939</v>
       </c>
       <c r="F14">
-        <v>0.3492264511841569</v>
+        <v>0.3547508176790478</v>
       </c>
     </row>
     <row r="15">
@@ -680,19 +680,19 @@
         </is>
       </c>
       <c r="B15">
-        <v>0.2529966507318655</v>
+        <v>0.2529966507318627</v>
       </c>
       <c r="C15">
-        <v>0.0005604785236366094</v>
+        <v>0.0006653036246888622</v>
       </c>
       <c r="D15">
-        <v>0.07333125665011515</v>
+        <v>0.07433443386871266</v>
       </c>
       <c r="E15">
-        <v>0.1092700287565765</v>
+        <v>0.1073038375380115</v>
       </c>
       <c r="F15">
-        <v>0.3967232727071545</v>
+        <v>0.3986894639257138</v>
       </c>
     </row>
     <row r="16">
@@ -702,19 +702,19 @@
         </is>
       </c>
       <c r="B16">
-        <v>0.2654588040080721</v>
+        <v>0.2654588040080677</v>
       </c>
       <c r="C16">
-        <v>0.0001834024825451142</v>
+        <v>0.000373479256535747</v>
       </c>
       <c r="D16">
-        <v>0.07096225372363414</v>
+        <v>0.07460589734746502</v>
       </c>
       <c r="E16">
-        <v>0.1263753424479559</v>
+        <v>0.119233932172744</v>
       </c>
       <c r="F16">
-        <v>0.4045422655681884</v>
+        <v>0.4116836758433914</v>
       </c>
     </row>
     <row r="17">
@@ -724,19 +724,19 @@
         </is>
       </c>
       <c r="B17">
-        <v>0.2752189661327938</v>
+        <v>0.2752189661327901</v>
       </c>
       <c r="C17">
-        <v>0.0002125609427707786</v>
+        <v>0.0003759190556591463</v>
       </c>
       <c r="D17">
-        <v>0.0743111921943226</v>
+        <v>0.07738615702192361</v>
       </c>
       <c r="E17">
-        <v>0.1295717057836876</v>
+        <v>0.1235448854678584</v>
       </c>
       <c r="F17">
-        <v>0.4208662264819001</v>
+        <v>0.4268930467977217</v>
       </c>
     </row>
     <row r="18">
@@ -746,19 +746,19 @@
         </is>
       </c>
       <c r="B18">
-        <v>0.09467851872762199</v>
+        <v>0.09467851872762714</v>
       </c>
       <c r="C18">
-        <v>0.4788880687052712</v>
+        <v>0.4722685068753598</v>
       </c>
       <c r="D18">
-        <v>0.1337093288898617</v>
+        <v>0.131718765104178</v>
       </c>
       <c r="E18">
-        <v>-0.1673869502935278</v>
+        <v>-0.1634855169646529</v>
       </c>
       <c r="F18">
-        <v>0.3567439877487719</v>
+        <v>0.3528425544199072</v>
       </c>
     </row>
     <row r="19">
@@ -768,19 +768,19 @@
         </is>
       </c>
       <c r="B19">
-        <v>0.2141789058785908</v>
+        <v>0.2141789058785948</v>
       </c>
       <c r="C19">
-        <v>0.0009301260147964729</v>
+        <v>0.0006628421289822661</v>
       </c>
       <c r="D19">
-        <v>0.06468997932296106</v>
+        <v>0.06291044911350566</v>
       </c>
       <c r="E19">
-        <v>0.08738887624494643</v>
+        <v>0.09087669136488397</v>
       </c>
       <c r="F19">
-        <v>0.3409689355122353</v>
+        <v>0.3374811203923056</v>
       </c>
     </row>
     <row r="20">
@@ -790,19 +790,19 @@
         </is>
       </c>
       <c r="B20">
-        <v>0.02416345094215887</v>
+        <v>0.02416345094216635</v>
       </c>
       <c r="C20">
-        <v>0.7433265738605133</v>
+        <v>0.7514619292334686</v>
       </c>
       <c r="D20">
-        <v>0.07379250347278553</v>
+        <v>0.07629464465809174</v>
       </c>
       <c r="E20">
-        <v>-0.1204671981935476</v>
+        <v>-0.1253713048009746</v>
       </c>
       <c r="F20">
-        <v>0.1687941000778653</v>
+        <v>0.1736982066853073</v>
       </c>
     </row>
     <row r="21">
@@ -812,19 +812,19 @@
         </is>
       </c>
       <c r="B21">
-        <v>0.2144724657361988</v>
+        <v>0.2144724657361956</v>
       </c>
       <c r="C21">
-        <v>0.0005237389541916659</v>
+        <v>0.0007727803186883264</v>
       </c>
       <c r="D21">
-        <v>0.06183770935026483</v>
+        <v>0.06378620265176761</v>
       </c>
       <c r="E21">
-        <v>0.09327278252322403</v>
+        <v>0.08945380582815785</v>
       </c>
       <c r="F21">
-        <v>0.3356721489491736</v>
+        <v>0.3394911256442333</v>
       </c>
     </row>
     <row r="22">
@@ -834,19 +834,19 @@
         </is>
       </c>
       <c r="B22">
-        <v>-0.1227442073636477</v>
+        <v>-0.1227442073636331</v>
       </c>
       <c r="C22">
-        <v>0.3360727149511973</v>
+        <v>0.3445924409747321</v>
       </c>
       <c r="D22">
-        <v>0.1275988335181931</v>
+        <v>0.1298701655125862</v>
       </c>
       <c r="E22">
-        <v>-0.3728333255286285</v>
+        <v>-0.3772850544345578</v>
       </c>
       <c r="F22">
-        <v>0.127344910801333</v>
+        <v>0.1317966397072916</v>
       </c>
     </row>
     <row r="23">
@@ -856,19 +856,19 @@
         </is>
       </c>
       <c r="B23">
-        <v>-0.08598698641499584</v>
+        <v>-0.08598698641497697</v>
       </c>
       <c r="C23">
-        <v>0.4028107899278486</v>
+        <v>0.41613508086606</v>
       </c>
       <c r="D23">
-        <v>0.1027800260890425</v>
+        <v>0.1057462254324677</v>
       </c>
       <c r="E23">
-        <v>-0.2874321358796062</v>
+        <v>-0.2932457797636671</v>
       </c>
       <c r="F23">
-        <v>0.1154581630496145</v>
+        <v>0.1212718069337131</v>
       </c>
     </row>
     <row r="24">
@@ -878,19 +878,19 @@
         </is>
       </c>
       <c r="B24">
-        <v>-0.1121040621674715</v>
+        <v>-0.1121040621674693</v>
       </c>
       <c r="C24">
-        <v>0.2804099790040659</v>
+        <v>0.2800065187264629</v>
       </c>
       <c r="D24">
-        <v>0.1038578703402321</v>
+        <v>0.1037707810237249</v>
       </c>
       <c r="E24">
-        <v>-0.315661747545357</v>
+        <v>-0.3154910556215624</v>
       </c>
       <c r="F24">
-        <v>0.09145362321041399</v>
+        <v>0.09128293128662388</v>
       </c>
     </row>
     <row r="25">
@@ -900,19 +900,19 @@
         </is>
       </c>
       <c r="B25">
-        <v>0.06642522617590131</v>
+        <v>0.06642522617590337</v>
       </c>
       <c r="C25">
-        <v>0.4557058308591446</v>
+        <v>0.4491011656066468</v>
       </c>
       <c r="D25">
-        <v>0.08904944912877881</v>
+        <v>0.08775791398322491</v>
       </c>
       <c r="E25">
-        <v>-0.1081084869596368</v>
+        <v>-0.1055771245895814</v>
       </c>
       <c r="F25">
-        <v>0.2409589393114394</v>
+        <v>0.2384275769413881</v>
       </c>
     </row>
     <row r="26">
@@ -922,19 +922,19 @@
         </is>
       </c>
       <c r="B26">
-        <v>0.1382687003678992</v>
+        <v>0.1382687003679039</v>
       </c>
       <c r="C26">
-        <v>0.1664176225567806</v>
+        <v>0.1567292153636706</v>
       </c>
       <c r="D26">
-        <v>0.09991907908825116</v>
+        <v>0.09763648470405195</v>
       </c>
       <c r="E26">
-        <v>-0.05756909601348226</v>
+        <v>-0.05309529322913373</v>
       </c>
       <c r="F26">
-        <v>0.3341064967492807</v>
+        <v>0.3296326939649415</v>
       </c>
     </row>
     <row r="27">
@@ -944,19 +944,19 @@
         </is>
       </c>
       <c r="B27">
-        <v>-0.06357971299271589</v>
+        <v>-0.06357971299270949</v>
       </c>
       <c r="C27">
-        <v>0.5102179617306719</v>
+        <v>0.4638895071741875</v>
       </c>
       <c r="D27">
-        <v>0.09655257862692175</v>
+        <v>0.08680330522665239</v>
       </c>
       <c r="E27">
-        <v>-0.2528192897159542</v>
+        <v>-0.2337110649759855</v>
       </c>
       <c r="F27">
-        <v>0.1256598637305225</v>
+        <v>0.1065516389905666</v>
       </c>
     </row>
     <row r="28">
@@ -966,19 +966,19 @@
         </is>
       </c>
       <c r="B28">
-        <v>0.02177717580227451</v>
+        <v>0.02177717580227423</v>
       </c>
       <c r="C28">
-        <v>0.761947076327925</v>
+        <v>0.7618194089661716</v>
       </c>
       <c r="D28">
-        <v>0.07188967975087963</v>
+        <v>0.07184994518523953</v>
       </c>
       <c r="E28">
-        <v>-0.1191240073695679</v>
+        <v>-0.1190461290519723</v>
       </c>
       <c r="F28">
-        <v>0.1626783589741169</v>
+        <v>0.1626004806565207</v>
       </c>
     </row>
     <row r="29">
@@ -988,19 +988,19 @@
         </is>
       </c>
       <c r="B29">
-        <v>0.0308492499123819</v>
+        <v>0.0308492499123776</v>
       </c>
       <c r="C29">
-        <v>0.7310897575766924</v>
+        <v>0.7330395429997236</v>
       </c>
       <c r="D29">
-        <v>0.08976252485761867</v>
+        <v>0.09044444607149525</v>
       </c>
       <c r="E29">
-        <v>-0.145082065969932</v>
+        <v>-0.1464186069894282</v>
       </c>
       <c r="F29">
-        <v>0.2067805657946958</v>
+        <v>0.2081171068141834</v>
       </c>
     </row>
     <row r="30">
@@ -1010,19 +1010,19 @@
         </is>
       </c>
       <c r="B30">
-        <v>-0.1333974708860022</v>
+        <v>-0.1333974708859983</v>
       </c>
       <c r="C30">
-        <v>0.1305755910570199</v>
+        <v>0.1484589296281091</v>
       </c>
       <c r="D30">
-        <v>0.08823541159263681</v>
+        <v>0.09231682630124319</v>
       </c>
       <c r="E30">
-        <v>-0.3063356997686383</v>
+        <v>-0.3143351256034749</v>
       </c>
       <c r="F30">
-        <v>0.0395407579966339</v>
+        <v>0.04754018383147829</v>
       </c>
     </row>
     <row r="31">
@@ -1032,19 +1032,19 @@
         </is>
       </c>
       <c r="B31">
-        <v>-0.1150517653242471</v>
+        <v>-0.1150517653242422</v>
       </c>
       <c r="C31">
-        <v>0.1917098915852897</v>
+        <v>0.2038404575230519</v>
       </c>
       <c r="D31">
-        <v>0.08812597617530385</v>
+        <v>0.09054304960162572</v>
       </c>
       <c r="E31">
-        <v>-0.2877755047302774</v>
+        <v>-0.2925128815938522</v>
       </c>
       <c r="F31">
-        <v>0.05767197408178326</v>
+        <v>0.06240935094536786</v>
       </c>
     </row>
     <row r="32">
@@ -1054,19 +1054,19 @@
         </is>
       </c>
       <c r="B32">
-        <v>-0.08963581965677622</v>
+        <v>-0.08963581965677316</v>
       </c>
       <c r="C32">
-        <v>0.3259778031539433</v>
+        <v>0.3060811250400122</v>
       </c>
       <c r="D32">
-        <v>0.09125581467220145</v>
+        <v>0.08757948551303392</v>
       </c>
       <c r="E32">
-        <v>-0.2684939297941529</v>
+        <v>-0.261288457046867</v>
       </c>
       <c r="F32">
-        <v>0.0892222904806004</v>
+        <v>0.08201681773332069</v>
       </c>
     </row>
     <row r="33">
@@ -1076,19 +1076,19 @@
         </is>
       </c>
       <c r="B33">
-        <v>-0.2478076138347083</v>
+        <v>-0.2478076138347055</v>
       </c>
       <c r="C33">
-        <v>0.01601476915885636</v>
+        <v>0.02015710058866915</v>
       </c>
       <c r="D33">
-        <v>0.1028854090495936</v>
+        <v>0.1066568279596284</v>
       </c>
       <c r="E33">
-        <v>-0.4494593101065831</v>
+        <v>-0.4568511553408618</v>
       </c>
       <c r="F33">
-        <v>-0.04615591756283349</v>
+        <v>-0.03876407232854917</v>
       </c>
     </row>
     <row r="34">
@@ -1098,19 +1098,19 @@
         </is>
       </c>
       <c r="B34">
-        <v>-0.07869898506363539</v>
+        <v>-0.07869898506362617</v>
       </c>
       <c r="C34">
-        <v>0.3778118838295756</v>
+        <v>0.3522613069413973</v>
       </c>
       <c r="D34">
-        <v>0.08923443646711146</v>
+        <v>0.0846032746316754</v>
       </c>
       <c r="E34">
-        <v>-0.2535952667199014</v>
+        <v>-0.2445183563158611</v>
       </c>
       <c r="F34">
-        <v>0.09619729659263064</v>
+        <v>0.08712038618860875</v>
       </c>
     </row>
     <row r="35">
@@ -1120,19 +1120,19 @@
         </is>
       </c>
       <c r="B35">
-        <v>-0.04120988995199463</v>
+        <v>-0.04120988995199227</v>
       </c>
       <c r="C35">
-        <v>0.7057767114307536</v>
+        <v>0.6902888004670276</v>
       </c>
       <c r="D35">
-        <v>0.109155404866632</v>
+        <v>0.1034220798970251</v>
       </c>
       <c r="E35">
-        <v>-0.2551505522084814</v>
+        <v>-0.2439134417563854</v>
       </c>
       <c r="F35">
-        <v>0.1727307723044921</v>
+        <v>0.1614936618524008</v>
       </c>
     </row>
     <row r="36">
@@ -1142,19 +1142,19 @@
         </is>
       </c>
       <c r="B36">
-        <v>0.1067126873633476</v>
+        <v>0.1067126873633552</v>
       </c>
       <c r="C36">
-        <v>0.2237789775716388</v>
+        <v>0.2175668352635023</v>
       </c>
       <c r="D36">
-        <v>0.08771813252969865</v>
+        <v>0.08654551183909864</v>
       </c>
       <c r="E36">
-        <v>-0.06521169318597307</v>
+        <v>-0.062913398864863</v>
       </c>
       <c r="F36">
-        <v>0.2786370679126682</v>
+        <v>0.2763387735915733</v>
       </c>
     </row>
     <row r="37">
@@ -1164,19 +1164,19 @@
         </is>
       </c>
       <c r="B37">
-        <v>-0.08032468614179963</v>
+        <v>-0.08032468614179283</v>
       </c>
       <c r="C37">
-        <v>0.4876330538894853</v>
+        <v>0.479202434302644</v>
       </c>
       <c r="D37">
-        <v>0.115728551746297</v>
+        <v>0.1135193380772947</v>
       </c>
       <c r="E37">
-        <v>-0.3071484795475217</v>
+        <v>-0.3028185003221167</v>
       </c>
       <c r="F37">
-        <v>0.1464991072639225</v>
+        <v>0.142169128038531</v>
       </c>
     </row>
     <row r="38">
@@ -1186,19 +1186,19 @@
         </is>
       </c>
       <c r="B38">
-        <v>-0.07688920420414269</v>
+        <v>-0.07688920420413223</v>
       </c>
       <c r="C38">
-        <v>0.4717534945626507</v>
+        <v>0.4776512210124535</v>
       </c>
       <c r="D38">
-        <v>0.1068456268998943</v>
+        <v>0.1082816397227158</v>
       </c>
       <c r="E38">
-        <v>-0.2863027848335395</v>
+        <v>-0.2891173182475969</v>
       </c>
       <c r="F38">
-        <v>0.1325243764252541</v>
+        <v>0.1353389098393324</v>
       </c>
     </row>
     <row r="39">
@@ -1208,19 +1208,19 @@
         </is>
       </c>
       <c r="B39">
-        <v>-0.09977871290359812</v>
+        <v>-0.09977871290359308</v>
       </c>
       <c r="C39">
-        <v>0.3914480769394322</v>
+        <v>0.3729838190964712</v>
       </c>
       <c r="D39">
-        <v>0.1164286877814139</v>
+        <v>0.1119978913425289</v>
       </c>
       <c r="E39">
-        <v>-0.3279747477224279</v>
+        <v>-0.31929054627938</v>
       </c>
       <c r="F39">
-        <v>0.1284173219152316</v>
+        <v>0.1197331204721938</v>
       </c>
     </row>
     <row r="40">
@@ -1230,19 +1230,19 @@
         </is>
       </c>
       <c r="B40">
-        <v>0.05670628474738666</v>
+        <v>0.05670628474738907</v>
       </c>
       <c r="C40">
-        <v>0.6232317279825719</v>
+        <v>0.6213689044196857</v>
       </c>
       <c r="D40">
-        <v>0.1154266897164683</v>
+        <v>0.1148106914296425</v>
       </c>
       <c r="E40">
-        <v>-0.1695258699515709</v>
+        <v>-0.1683185354948516</v>
       </c>
       <c r="F40">
-        <v>0.2829384394463442</v>
+        <v>0.2817311049896298</v>
       </c>
     </row>
     <row r="41">
@@ -1252,19 +1252,19 @@
         </is>
       </c>
       <c r="B41">
-        <v>0.1744026195933822</v>
+        <v>0.1744026195933864</v>
       </c>
       <c r="C41">
-        <v>0.06750215177270413</v>
+        <v>0.07286569045550184</v>
       </c>
       <c r="D41">
-        <v>0.09538976147704374</v>
+        <v>0.09723222140639935</v>
       </c>
       <c r="E41">
-        <v>-0.01255787739548977</v>
+        <v>-0.01616903249998078</v>
       </c>
       <c r="F41">
-        <v>0.3613631165822541</v>
+        <v>0.3649742716867536</v>
       </c>
     </row>
     <row r="42">
@@ -1274,19 +1274,19 @@
         </is>
       </c>
       <c r="B42">
-        <v>-0.1352749227840047</v>
+        <v>-0.1352749227839941</v>
       </c>
       <c r="C42">
-        <v>0.2120948245907819</v>
+        <v>0.2204706172953215</v>
       </c>
       <c r="D42">
-        <v>0.108408491656729</v>
+        <v>0.1104034829343153</v>
       </c>
       <c r="E42">
-        <v>-0.3477516620495045</v>
+        <v>-0.3516617731030345</v>
       </c>
       <c r="F42">
-        <v>0.0772018164814951</v>
+        <v>0.0811119275350464</v>
       </c>
     </row>
     <row r="43">
@@ -1296,19 +1296,19 @@
         </is>
       </c>
       <c r="B43">
-        <v>0.01008256803722173</v>
+        <v>0.01008256803722867</v>
       </c>
       <c r="C43">
-        <v>0.9406794335359827</v>
+        <v>0.9406994902733694</v>
       </c>
       <c r="D43">
-        <v>0.1354893773334267</v>
+        <v>0.1355352874917078</v>
       </c>
       <c r="E43">
-        <v>-0.255471731824052</v>
+        <v>-0.2555617140808006</v>
       </c>
       <c r="F43">
-        <v>0.2756368678984955</v>
+        <v>0.275726850155258</v>
       </c>
     </row>
     <row r="44">
@@ -1318,19 +1318,19 @@
         </is>
       </c>
       <c r="B44">
-        <v>0.1926714109760419</v>
+        <v>0.1926714109760423</v>
       </c>
       <c r="C44">
-        <v>0.09532562304214665</v>
+        <v>0.07581139188807051</v>
       </c>
       <c r="D44">
-        <v>0.1155138904941029</v>
+        <v>0.1085152335073855</v>
       </c>
       <c r="E44">
-        <v>-0.0337316541065035</v>
+        <v>-0.02001453847238724</v>
       </c>
       <c r="F44">
-        <v>0.4190744760585873</v>
+        <v>0.4053573604244718</v>
       </c>
     </row>
     <row r="45">
@@ -1340,19 +1340,19 @@
         </is>
       </c>
       <c r="B45">
-        <v>-0.1153070969394708</v>
+        <v>-0.1153070969394807</v>
       </c>
       <c r="C45">
-        <v>0.3202777006762576</v>
+        <v>0.3651755093749203</v>
       </c>
       <c r="D45">
-        <v>0.1160162606515062</v>
+        <v>0.1273341502606303</v>
       </c>
       <c r="E45">
-        <v>-0.3426947894374343</v>
+        <v>-0.3648774454523275</v>
       </c>
       <c r="F45">
-        <v>0.1120805955584926</v>
+        <v>0.1342632515733661</v>
       </c>
     </row>
     <row r="46">
@@ -1362,19 +1362,19 @@
         </is>
       </c>
       <c r="B46">
-        <v>-0.04781844856425704</v>
+        <v>-0.0478184485642535</v>
       </c>
       <c r="C46">
-        <v>0.6829138280984095</v>
+        <v>0.6832712850500542</v>
       </c>
       <c r="D46">
-        <v>0.1170614355859063</v>
+        <v>0.1172011447314192</v>
       </c>
       <c r="E46">
-        <v>-0.2772546462911887</v>
+        <v>-0.2775284711847013</v>
       </c>
       <c r="F46">
-        <v>0.1816177491626746</v>
+        <v>0.1818915740561943</v>
       </c>
     </row>
     <row r="47">
@@ -1384,19 +1384,19 @@
         </is>
       </c>
       <c r="B47">
-        <v>-0.2490495787445668</v>
+        <v>-0.2490495787445562</v>
       </c>
       <c r="C47">
-        <v>0.04835487612235001</v>
+        <v>0.03834055330225827</v>
       </c>
       <c r="D47">
-        <v>0.1261498302891022</v>
+        <v>0.1202443751821547</v>
       </c>
       <c r="E47">
-        <v>-0.4962987027670471</v>
+        <v>-0.4847242234451013</v>
       </c>
       <c r="F47">
-        <v>-0.001800454722086481</v>
+        <v>-0.01337493404401113</v>
       </c>
     </row>
     <row r="48">
@@ -1406,19 +1406,19 @@
         </is>
       </c>
       <c r="B48">
-        <v>0.01645486145732713</v>
+        <v>0.01645486145734172</v>
       </c>
       <c r="C48">
-        <v>0.8847774226516281</v>
+        <v>0.8849801990555937</v>
       </c>
       <c r="D48">
-        <v>0.113547809736308</v>
+        <v>0.1137493970175264</v>
       </c>
       <c r="E48">
-        <v>-0.2060947561492431</v>
+        <v>-0.2064898599601578</v>
       </c>
       <c r="F48">
-        <v>0.2390044790638973</v>
+        <v>0.2393995828748413</v>
       </c>
     </row>
     <row r="49">
@@ -1428,19 +1428,19 @@
         </is>
       </c>
       <c r="B49">
-        <v>0.01742405879954825</v>
+        <v>0.01742405879953857</v>
       </c>
       <c r="C49">
-        <v>0.8817204400057925</v>
+        <v>0.8814223075375853</v>
       </c>
       <c r="D49">
-        <v>0.11710613482746</v>
+        <v>0.1168095170370898</v>
       </c>
       <c r="E49">
-        <v>-0.2120997478309649</v>
+        <v>-0.2115183876446752</v>
       </c>
       <c r="F49">
-        <v>0.2469478654300614</v>
+        <v>0.2463665052437523</v>
       </c>
     </row>
     <row r="50">
@@ -1450,19 +1450,19 @@
         </is>
       </c>
       <c r="B50">
-        <v>0.1076066077090127</v>
+        <v>0.1076066077090035</v>
       </c>
       <c r="C50">
-        <v>0.4798282679626638</v>
+        <v>0.4635340809115616</v>
       </c>
       <c r="D50">
-        <v>0.1522924376890555</v>
+        <v>0.1467950169199711</v>
       </c>
       <c r="E50">
-        <v>-0.1908810852793463</v>
+        <v>-0.1801063385640877</v>
       </c>
       <c r="F50">
-        <v>0.4060943006973716</v>
+        <v>0.3953195539820946</v>
       </c>
     </row>
     <row r="51">
@@ -1472,19 +1472,19 @@
         </is>
       </c>
       <c r="B51">
-        <v>-0.08420136588236431</v>
+        <v>-0.08420136588235551</v>
       </c>
       <c r="C51">
-        <v>0.5015352982581871</v>
+        <v>0.4990062576306764</v>
       </c>
       <c r="D51">
-        <v>0.1252854776676644</v>
+        <v>0.1245482544947847</v>
       </c>
       <c r="E51">
-        <v>-0.3297563898968837</v>
+        <v>-0.3283114590294624</v>
       </c>
       <c r="F51">
-        <v>0.1613536581321551</v>
+        <v>0.1599087272647514</v>
       </c>
     </row>
     <row r="52">
@@ -1494,19 +1494,19 @@
         </is>
       </c>
       <c r="B52">
-        <v>0.03290842845463285</v>
+        <v>0.03290842845463741</v>
       </c>
       <c r="C52">
-        <v>0.8022693434444248</v>
+        <v>0.8053492271647535</v>
       </c>
       <c r="D52">
-        <v>0.1314175407872173</v>
+        <v>0.133540563801817</v>
       </c>
       <c r="E52">
-        <v>-0.2246652184251365</v>
+        <v>-0.228826267072097</v>
       </c>
       <c r="F52">
-        <v>0.2904820753344022</v>
+        <v>0.2946431239813718</v>
       </c>
     </row>
     <row r="53">
@@ -1516,19 +1516,19 @@
         </is>
       </c>
       <c r="B53">
-        <v>-0.3199884550045603</v>
+        <v>-0.319988455004551</v>
       </c>
       <c r="C53">
-        <v>0.005206396557691395</v>
+        <v>0.004488050433350876</v>
       </c>
       <c r="D53">
-        <v>0.1145278938916254</v>
+        <v>0.112606503894583</v>
       </c>
       <c r="E53">
-        <v>-0.5444590022573709</v>
+        <v>-0.5406931470629029</v>
       </c>
       <c r="F53">
-        <v>-0.09551790775174973</v>
+        <v>-0.09928376294619909</v>
       </c>
     </row>
     <row r="54">
@@ -1538,19 +1538,19 @@
         </is>
       </c>
       <c r="B54">
-        <v>-1.436021072955095</v>
+        <v>-1.436021072955121</v>
       </c>
       <c r="C54">
-        <v>0.00195055818840939</v>
+        <v>0.00153598723608428</v>
       </c>
       <c r="D54">
-        <v>0.4635827042319545</v>
+        <v>0.4533185259689707</v>
       </c>
       <c r="E54">
-        <v>-2.34462647710541</v>
+        <v>-2.324509057379089</v>
       </c>
       <c r="F54">
-        <v>-0.5274156688047806</v>
+        <v>-0.5475330885311539</v>
       </c>
     </row>
     <row r="55">
@@ -1560,19 +1560,19 @@
         </is>
       </c>
       <c r="B55">
-        <v>-2.006554496392117</v>
+        <v>-2.006554496392113</v>
       </c>
       <c r="C55">
-        <v>0.02265478200945426</v>
+        <v>0.01830434786352475</v>
       </c>
       <c r="D55">
-        <v>0.8803740841786009</v>
+        <v>0.850449962113468</v>
       </c>
       <c r="E55">
-        <v>-3.732055994304607</v>
+        <v>-3.673405792787963</v>
       </c>
       <c r="F55">
-        <v>-0.2810529984796257</v>
+        <v>-0.3397031999962625</v>
       </c>
     </row>
     <row r="56">
@@ -1582,19 +1582,19 @@
         </is>
       </c>
       <c r="B56">
-        <v>-1.62807619826694</v>
+        <v>-1.628076198266907</v>
       </c>
       <c r="C56">
-        <v>0.1103603660737853</v>
+        <v>0.1177416456765081</v>
       </c>
       <c r="D56">
-        <v>1.019730171713425</v>
+        <v>1.040754249199942</v>
       </c>
       <c r="E56">
-        <v>-3.626710608774098</v>
+        <v>-3.667917043455816</v>
       </c>
       <c r="F56">
-        <v>0.3705582122402178</v>
+        <v>0.4117646469220018</v>
       </c>
     </row>
     <row r="57">
@@ -1604,19 +1604,19 @@
         </is>
       </c>
       <c r="B57">
-        <v>-1.363088172843181</v>
+        <v>-1.363088172843142</v>
       </c>
       <c r="C57">
-        <v>0.205971614787837</v>
+        <v>0.2153103415066531</v>
       </c>
       <c r="D57">
-        <v>1.077778372253707</v>
+        <v>1.100067582608667</v>
       </c>
       <c r="E57">
-        <v>-3.475494965776648</v>
+        <v>-3.519181015316168</v>
       </c>
       <c r="F57">
-        <v>0.7493186200902873</v>
+        <v>0.7930046696298854</v>
       </c>
     </row>
     <row r="58">
@@ -1626,19 +1626,19 @@
         </is>
       </c>
       <c r="B58">
-        <v>-2.056481448812635</v>
+        <v>-2.056481448812628</v>
       </c>
       <c r="C58">
-        <v>0.07230893849902698</v>
+        <v>0.06497423122014023</v>
       </c>
       <c r="D58">
-        <v>1.144289985204588</v>
+        <v>1.114361129487362</v>
       </c>
       <c r="E58">
-        <v>-4.299248607683499</v>
+        <v>-4.240589128379233</v>
       </c>
       <c r="F58">
-        <v>0.1862857100582276</v>
+        <v>0.1276262307539757</v>
       </c>
     </row>
     <row r="59">
@@ -1648,19 +1648,19 @@
         </is>
       </c>
       <c r="B59">
-        <v>-2.233550538525456</v>
+        <v>-2.23355053852546</v>
       </c>
       <c r="C59">
-        <v>0.0371383481758405</v>
+        <v>0.03069704504355797</v>
       </c>
       <c r="D59">
-        <v>1.071637916769098</v>
+        <v>1.033583229894412</v>
       </c>
       <c r="E59">
-        <v>-4.33392225986042</v>
+        <v>-4.25933644414309</v>
       </c>
       <c r="F59">
-        <v>-0.1331788171904931</v>
+        <v>-0.2077646329078302</v>
       </c>
     </row>
     <row r="60">
@@ -1670,19 +1670,19 @@
         </is>
       </c>
       <c r="B60">
-        <v>-2.084809423381722</v>
+        <v>-2.0848094233817</v>
       </c>
       <c r="C60">
-        <v>0.05405076422374533</v>
+        <v>0.04857109707929719</v>
       </c>
       <c r="D60">
-        <v>1.082214220781883</v>
+        <v>1.057024710770205</v>
       </c>
       <c r="E60">
-        <v>-4.20591031967129</v>
+        <v>-4.156539787260169</v>
       </c>
       <c r="F60">
-        <v>0.03629147290784651</v>
+        <v>-0.01307905950323152</v>
       </c>
     </row>
     <row r="61">
@@ -1692,19 +1692,19 @@
         </is>
       </c>
       <c r="B61">
-        <v>-1.755404378560876</v>
+        <v>-1.755404378560845</v>
       </c>
       <c r="C61">
-        <v>0.1370091076385558</v>
+        <v>0.1458699493404563</v>
       </c>
       <c r="D61">
-        <v>1.180483447625576</v>
+        <v>1.207064561382327</v>
       </c>
       <c r="E61">
-        <v>-4.06910942025268</v>
+        <v>-4.121207445884843</v>
       </c>
       <c r="F61">
-        <v>0.5583006631309275</v>
+        <v>0.6103986887631534</v>
       </c>
     </row>
     <row r="62">
@@ -1714,19 +1714,19 @@
         </is>
       </c>
       <c r="B62">
-        <v>-2.105443960167777</v>
+        <v>-2.105443960167747</v>
       </c>
       <c r="C62">
-        <v>0.07696595467992107</v>
+        <v>0.08280218770821324</v>
       </c>
       <c r="D62">
-        <v>1.190479344547652</v>
+        <v>1.213754732623231</v>
       </c>
       <c r="E62">
-        <v>-4.438740599820024</v>
+        <v>-4.484359522174323</v>
       </c>
       <c r="F62">
-        <v>0.2278526794844704</v>
+        <v>0.2734716018388279</v>
       </c>
     </row>
     <row r="63">
@@ -1736,19 +1736,19 @@
         </is>
       </c>
       <c r="B63">
-        <v>-2.546142172309576</v>
+        <v>-2.546142172309544</v>
       </c>
       <c r="C63">
-        <v>0.04329093781589521</v>
+        <v>0.0417682549223839</v>
       </c>
       <c r="D63">
-        <v>1.259910014922015</v>
+        <v>1.250670467268978</v>
       </c>
       <c r="E63">
-        <v>-5.015520425318048</v>
+        <v>-4.997411244684621</v>
       </c>
       <c r="F63">
-        <v>-0.07676391930110382</v>
+        <v>-0.09487309993446669</v>
       </c>
     </row>
     <row r="64">
@@ -1758,19 +1758,19 @@
         </is>
       </c>
       <c r="B64">
-        <v>-2.187699511178846</v>
+        <v>-2.187699511178809</v>
       </c>
       <c r="C64">
-        <v>0.06805303532399187</v>
+        <v>0.06727602705205094</v>
       </c>
       <c r="D64">
-        <v>1.198965795768775</v>
+        <v>1.195578177378444</v>
       </c>
       <c r="E64">
-        <v>-4.53762928958105</v>
+        <v>-4.5309896795426</v>
       </c>
       <c r="F64">
-        <v>0.1622302672233582</v>
+        <v>0.1555906571849808</v>
       </c>
     </row>
     <row r="65">
@@ -1780,19 +1780,19 @@
         </is>
       </c>
       <c r="B65">
-        <v>-0.7983840708842894</v>
+        <v>-0.798384070884269</v>
       </c>
       <c r="C65">
-        <v>0.3279249210698167</v>
+        <v>0.3523834851468415</v>
       </c>
       <c r="D65">
-        <v>0.8160915258302519</v>
+        <v>0.8584996044967611</v>
       </c>
       <c r="E65">
-        <v>-2.397894069599922</v>
+        <v>-2.481012376439801</v>
       </c>
       <c r="F65">
-        <v>0.8011259278313431</v>
+        <v>0.8842442346712628</v>
       </c>
     </row>
     <row r="66">
@@ -1802,19 +1802,19 @@
         </is>
       </c>
       <c r="B66">
-        <v>0.1109111489083722</v>
+        <v>0.110911148908075</v>
       </c>
       <c r="C66">
-        <v>0.7020826135722673</v>
+        <v>0.7058107918718366</v>
       </c>
       <c r="D66">
-        <v>0.2899556970400872</v>
+        <v>0.2938135101088578</v>
       </c>
       <c r="E66">
-        <v>-0.4573915744024056</v>
+        <v>-0.464952749076581</v>
       </c>
       <c r="F66">
-        <v>0.6792138722191501</v>
+        <v>0.6867750468927312</v>
       </c>
     </row>
   </sheetData>
@@ -1866,19 +1866,19 @@
         </is>
       </c>
       <c r="B2">
-        <v>-1.824915224457785</v>
+        <v>-1.824915224457771</v>
       </c>
       <c r="C2">
-        <v>0.06273348413159008</v>
+        <v>0.06147650068927479</v>
       </c>
       <c r="D2">
-        <v>0.9805701093946699</v>
+        <v>0.975862995553026</v>
       </c>
       <c r="E2">
-        <v>-3.746797323187838</v>
+        <v>-3.737571549587072</v>
       </c>
       <c r="F2">
-        <v>0.09696687427226869</v>
+        <v>0.08774110067153051</v>
       </c>
     </row>
   </sheetData>

</xml_diff>